<commit_message>
Update CDIFcompleteProfile schema, fix CI workflow paths, update property workbooks
- Restructure CDIFcompleteProfile to compose via allOf with 4 BB refs
- Add explicit conformsTo contains constraints for all 4 component URIs
- Fix update-validation-schemas workflow: use Profile suffix in paths
- Fix cdi:physicalDataType string→array in CDIFcomplete example
- Regenerate property workbooks with propertyTree worksheets
- Add add_property_tree.py tool for Excel propertyTree generation

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_sources/cdifProperties/cdifCore/cdifCore_properties.xlsx
+++ b/_sources/cdifProperties/cdifCore/cdifCore_properties.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/944a82e2ddcde9eb/Documents/GithubC/CDIF/metadataBuildingBlocksFork/_sources/cdifProperties/cdifCore/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="11_05052B09E4C4201FDF7C04F5839C58910C8DF9A7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC2D4775-7F23-4307-B503-5A9955565D35}"/>
+  <xr:revisionPtr revIDLastSave="202" documentId="11_05052B09E4C4201FDF7C04F5839C58910C8DF9A7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A91D89B7-0539-412E-B719-E6857151C2C8}"/>
   <bookViews>
-    <workbookView xWindow="1875" yWindow="390" windowWidth="22080" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4380" yWindow="525" windowWidth="21825" windowHeight="16020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="9" r:id="rId1"/>
+    <sheet name="propertyTree" sheetId="9" r:id="rId1"/>
     <sheet name="cdifCore" sheetId="1" r:id="rId2"/>
     <sheet name="identifier" sheetId="2" r:id="rId3"/>
     <sheet name="labeledLink" sheetId="3" r:id="rId4"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="172">
   <si>
     <t>Field Name</t>
   </si>
@@ -173,9 +173,6 @@
     <t>Distribution object</t>
   </si>
   <si>
-    <t>array of dataDownload</t>
-  </si>
-  <si>
     <t>0..* (required if no schema:url)</t>
   </si>
   <si>
@@ -482,7 +479,88 @@
     <t>Schema:Dataset</t>
   </si>
   <si>
-    <t>@type  identifier</t>
+    <t>string(date)</t>
+  </si>
+  <si>
+    <t>identifier</t>
+  </si>
+  <si>
+    <t>[string]</t>
+  </si>
+  <si>
+    <t>[object reference]</t>
+  </si>
+  <si>
+    <t>[labeledLink]</t>
+  </si>
+  <si>
+    <t>string (URI)</t>
+  </si>
+  <si>
+    <t>array of dataDownload | WebAPI</t>
+  </si>
+  <si>
+    <t>[DataDownload]</t>
+  </si>
+  <si>
+    <t>string(uri)</t>
+  </si>
+  <si>
+    <t>algorithm</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>person</t>
+  </si>
+  <si>
+    <t>[person]</t>
+  </si>
+  <si>
+    <t>[organization]</t>
+  </si>
+  <si>
+    <t>[WebAPI]</t>
+  </si>
+  <si>
+    <t>schema:serviceType</t>
+  </si>
+  <si>
+    <t>schema:termsOfService</t>
+  </si>
+  <si>
+    <t>schema:documentation</t>
+  </si>
+  <si>
+    <t>schema:potentialAction</t>
+  </si>
+  <si>
+    <t>[Action]</t>
+  </si>
+  <si>
+    <t>definedTerm</t>
+  </si>
+  <si>
+    <t>LabeledLink</t>
+  </si>
+  <si>
+    <t>cdifCatalogRecord</t>
+  </si>
+  <si>
+    <t>DataCatalog</t>
+  </si>
+  <si>
+    <t>property</t>
+  </si>
+  <si>
+    <t>object/data type</t>
+  </si>
+  <si>
+    <t>spdx:Checksum</t>
+  </si>
+  <si>
+    <t>object/datatype</t>
   </si>
 </sst>
 </file>
@@ -529,7 +607,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -538,6 +616,11 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,6 +636,92 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>581025</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8577AF0C-C6FC-1164-352A-A7D7BA5C8CA3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10115550" y="762000"/>
+          <a:ext cx="2714625" cy="1333500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100"/>
+            <a:t>[..]</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t> -- value is an array (JSON list)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" baseline="0"/>
+            <a:t>object -- value is an object, properties not expanded here. </a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -840,117 +1009,531 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C0A965B-6F37-4258-BA81-43BF9A6AB2B3}">
-  <dimension ref="A4:D21"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" customWidth="1"/>
     <col min="2" max="2" width="30.85546875" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="28.7109375" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.140625" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F1" t="s">
+        <v>168</v>
+      </c>
+      <c r="G1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B8" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B9" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="2"/>
+      <c r="C8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="2"/>
+      <c r="C9" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B10" s="2"/>
-      <c r="C10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C10" s="3"/>
+      <c r="D10" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B11" s="2"/>
-      <c r="C11" s="3" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C11" s="3"/>
+      <c r="D11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B12" s="2"/>
       <c r="C12" s="3"/>
       <c r="D12" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="2"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="E12" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="2"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="2" t="s">
+      <c r="C14" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+      <c r="C17" t="s">
+        <v>147</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="2"/>
+      <c r="C18" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="2"/>
+      <c r="D19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="2"/>
+      <c r="D20" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D21" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="2" t="s">
+      <c r="E21" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" s="2" t="s">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23" s="2"/>
+      <c r="C23" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="2"/>
+      <c r="C24" t="s">
+        <v>147</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="2"/>
+      <c r="C25" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="2"/>
+      <c r="D26" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D27" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D28" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B20" s="2" t="s">
+      <c r="E28" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C29" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="2:2" ht="30" x14ac:dyDescent="0.25">
-      <c r="B21" s="2" t="s">
-        <v>49</v>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="2"/>
+      <c r="C31" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="2"/>
+      <c r="D32" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B33" s="2"/>
+      <c r="D33" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B34" s="2"/>
+      <c r="D34" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E34" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D35" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D36" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D37" s="2"/>
+      <c r="E37" s="2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F38" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="G38" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D39" s="2"/>
+      <c r="F39" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="G39" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D40" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D41" s="2"/>
+      <c r="E41" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D42" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E43" t="s">
+        <v>147</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G43" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E44" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G44" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E45" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="G45" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C46" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D47" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E47" s="2"/>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D48" s="2"/>
+      <c r="E48" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D49" s="2"/>
+      <c r="E49" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="G49" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D50" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E50" s="2"/>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D51" s="2"/>
+      <c r="E51" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D52" s="2"/>
+      <c r="E52" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G52" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D53" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D54" s="2"/>
+      <c r="E54" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D55" s="2"/>
+      <c r="E55" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G55" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D56" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="G56" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B58" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="C59" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D60" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D61" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D62" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D63" s="2"/>
+      <c r="E63" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G63" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="D64" s="2"/>
+      <c r="E64" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="G64" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="65" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="D65" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="66" spans="4:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D66" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="G66" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1178,24 +1761,24 @@
         <v>45</v>
       </c>
       <c r="D11" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>10</v>
@@ -1248,50 +1831,50 @@
         <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -1299,7 +1882,7 @@
         <v>39</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>40</v>
@@ -1308,10 +1891,10 @@
         <v>41</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1361,16 +1944,16 @@
         <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1378,7 +1961,7 @@
         <v>21</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>22</v>
@@ -1387,15 +1970,15 @@
         <v>14</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>6</v>
@@ -1404,7 +1987,7 @@
         <v>14</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -1412,7 +1995,7 @@
         <v>39</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>40</v>
@@ -1424,7 +2007,7 @@
         <v>10</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1474,13 +2057,13 @@
         <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -1488,7 +2071,7 @@
         <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>17</v>
@@ -1497,10 +2080,10 @@
         <v>18</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1508,7 +2091,7 @@
         <v>21</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>22</v>
@@ -1517,15 +2100,15 @@
         <v>14</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>6</v>
@@ -1534,18 +2117,18 @@
         <v>14</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>41</v>
@@ -1556,79 +2139,79 @@
     </row>
     <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>17</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>72</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>74</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>75</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>83</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1687,18 +2270,18 @@
         <v>18</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>17</v>
@@ -1707,10 +2290,10 @@
         <v>18</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -1727,32 +2310,32 @@
         <v>10</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>8</v>
@@ -1764,46 +2347,46 @@
         <v>18</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>8</v>
@@ -1812,13 +2395,13 @@
         <v>9</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1868,13 +2451,13 @@
         <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
@@ -1882,16 +2465,16 @@
         <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="60" x14ac:dyDescent="0.25">
@@ -1899,7 +2482,7 @@
         <v>21</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>22</v>
@@ -1908,18 +2491,18 @@
         <v>14</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>6</v>
@@ -1928,7 +2511,7 @@
         <v>14</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -1936,7 +2519,7 @@
         <v>24</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>25</v>
@@ -1945,84 +2528,84 @@
         <v>26</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>116</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>117</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>9</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F9" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>118</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -2072,13 +2655,13 @@
         <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -2086,39 +2669,39 @@
         <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="105" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>87</v>
-      </c>
       <c r="D4" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="60" x14ac:dyDescent="0.25">
@@ -2126,7 +2709,7 @@
         <v>21</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>22</v>
@@ -2135,35 +2718,35 @@
         <v>14</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>6</v>
@@ -2172,7 +2755,7 @@
         <v>14</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="45" x14ac:dyDescent="0.25">
@@ -2180,7 +2763,7 @@
         <v>24</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>25</v>
@@ -2189,27 +2772,27 @@
         <v>26</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>121</v>
-      </c>
       <c r="E9" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -2259,16 +2842,16 @@
         <v>16</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="90" x14ac:dyDescent="0.25">
@@ -2276,7 +2859,7 @@
         <v>21</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>22</v>
@@ -2285,10 +2868,10 @@
         <v>14</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="75" x14ac:dyDescent="0.25">
@@ -2296,53 +2879,53 @@
         <v>24</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>